<commit_message>
feat: restrict loaders to requested mapped signals
Agent-Logs-Url: https://github.com/ec0k1ng/smart_analyzer/sessions/242936f1-f0eb-436f-9231-b390d0313f60

Co-authored-by: ec0k1ng <273817871+ec0k1ng@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/tcs_smart_analyzer/config/interface_mapping.xlsx
+++ b/src/tcs_smart_analyzer/config/interface_mapping.xlsx
@@ -424,7 +424,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -471,7 +471,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>时间轴，单位 s，必须配置且固定排在第一行。</t>
+          <t>时间轴，单位 s。</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>